<commit_message>
Last of Evidence Generated
</commit_message>
<xml_diff>
--- a/Docs/Data/Data_Generation_Info.xlsx
+++ b/Docs/Data/Data_Generation_Info.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29426"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Allison\Documents\SFU\IntelliAudit - Documentation\Samples\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\allyftw\Documents\GitHub\IntelliAudit\Docs\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C97CF0A5-66A6-4E1D-AA73-046BCA98F117}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E8DE05AA-BA16-45C4-A909-13871D2B555A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5550" yWindow="1125" windowWidth="16485" windowHeight="12960" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Artifacts" sheetId="1" r:id="rId1"/>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="72" uniqueCount="58">
   <si>
     <t>Artifact</t>
   </si>
@@ -34,12 +34,6 @@
     <t>5-2_Org_Chart.pdf</t>
   </si>
   <si>
-    <t>Synthetic / Organic</t>
-  </si>
-  <si>
-    <t>Organic</t>
-  </si>
-  <si>
     <t>Synthetic</t>
   </si>
   <si>
@@ -70,9 +64,6 @@
     <t>A3</t>
   </si>
   <si>
-    <t>Please generate for me a NIST SP 800-61 Rev. 3 compliant incident response report.</t>
-  </si>
-  <si>
     <t>S2</t>
   </si>
   <si>
@@ -136,9 +127,6 @@
     <t>Information security, cybersecurity and privacy protection — Information security management systems — Requirements</t>
   </si>
   <si>
-    <t>A1, A2, S3</t>
-  </si>
-  <si>
     <t>This is the Information Security policy for the Provencal Government of British Columbia. Please adapt the Information Security policy to fit my organization and ensure it is compliant with NIST.SP.800-100. </t>
   </si>
   <si>
@@ -152,6 +140,66 @@
   </si>
   <si>
     <t>A1, A2, S1, S4</t>
+  </si>
+  <si>
+    <t>Attached is the NIST Standard for incident repose.  Please create for my org an Incident Management Policy in accordance with ISO27001 control 5-24.</t>
+  </si>
+  <si>
+    <t>5-24_Incident_Management_Policy.docx</t>
+  </si>
+  <si>
+    <t>A5</t>
+  </si>
+  <si>
+    <t>A6</t>
+  </si>
+  <si>
+    <t>A7</t>
+  </si>
+  <si>
+    <t>A8</t>
+  </si>
+  <si>
+    <t>I am trying to create examples of a three strike policy in action. Please create for me an email from Sarah Johnson (CISO) to Amanda Taylor (CHRO) documenting the fact that Sarah reprimanded Joseph Thomas (on the IT Operations team) for an Information Security Policy violation.</t>
+  </si>
+  <si>
+    <t>It seems that Joseph Thomas has once again violated policy. Please create a written warning for similar but difference violations of the Information Security Policy.</t>
+  </si>
+  <si>
+    <t>It seems Joseph Thomas is a problem employee and has for a third and final time violated the Information Security policy. Please generate a formal termination letter written from Amanda Taylor to Joseph Thomas.</t>
+  </si>
+  <si>
+    <t>A1, A2, S1, S5</t>
+  </si>
+  <si>
+    <t>A1, A2, S1, S3</t>
+  </si>
+  <si>
+    <t>6-4_Written_Warning.txt</t>
+  </si>
+  <si>
+    <t>6-4_Termination_Letter.txt</t>
+  </si>
+  <si>
+    <t>6-4_Verbal_Warning.txt</t>
+  </si>
+  <si>
+    <t>A1, A2, A6, S1, S5</t>
+  </si>
+  <si>
+    <t>A1, A2, A6, A7, S1, S5</t>
+  </si>
+  <si>
+    <t>Data Type</t>
+  </si>
+  <si>
+    <t>Real World</t>
+  </si>
+  <si>
+    <t>Attached is my Incident Management Policy and the NIST standard for incident response.  Please create for me an incident response report.</t>
+  </si>
+  <si>
+    <t>A1, A2, A4,  S1, S3, S5</t>
   </si>
 </sst>
 </file>
@@ -217,7 +265,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
@@ -228,6 +276,9 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -509,12 +560,12 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F11"/>
+  <dimension ref="A1:F12"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="38.7109375" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="19.85546875" customWidth="1"/>
-    <col min="4" max="4" width="18" customWidth="1"/>
+    <col min="4" max="4" width="19.42578125" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="12" customWidth="1"/>
     <col min="6" max="6" width="205.28515625" bestFit="1" customWidth="1"/>
   </cols>
@@ -529,11 +580,11 @@
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="6" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="B2" s="6"/>
       <c r="C2" s="5" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="D2" s="5"/>
       <c r="E2" s="5"/>
@@ -549,113 +600,179 @@
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="B4" s="3" t="s">
         <v>0</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>2</v>
+        <v>54</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>38</v>
+        <v>34</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="B5" s="2" t="s">
         <v>1</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>3</v>
+        <v>55</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="E5" s="2"/>
       <c r="F5" s="2" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="B6" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="C6" t="s">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D6" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="E6" t="s">
-        <v>39</v>
+        <v>35</v>
       </c>
       <c r="F6" t="s">
-        <v>37</v>
+        <v>33</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>40</v>
-      </c>
-      <c r="C7" s="2"/>
+        <v>36</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>2</v>
+      </c>
       <c r="D7" s="2" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>39</v>
+        <v>35</v>
       </c>
       <c r="F7" s="2"/>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="B8" t="s">
-        <v>22</v>
+        <v>39</v>
       </c>
       <c r="C8" t="s">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D8" t="s">
-        <v>36</v>
+        <v>48</v>
       </c>
       <c r="E8" t="s">
-        <v>39</v>
+        <v>35</v>
       </c>
       <c r="F8" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A9" s="2"/>
-      <c r="B9" s="2"/>
-      <c r="C9" s="2"/>
-      <c r="D9" s="2"/>
-      <c r="E9" s="2"/>
-      <c r="F9" s="2"/>
+        <v>38</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D9" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="E9" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="F9" s="2" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>41</v>
+      </c>
+      <c r="B10" t="s">
+        <v>51</v>
+      </c>
+      <c r="C10" t="s">
+        <v>2</v>
+      </c>
+      <c r="D10" t="s">
+        <v>47</v>
+      </c>
+      <c r="E10" t="s">
+        <v>35</v>
+      </c>
+      <c r="F10" s="7" t="s">
+        <v>44</v>
+      </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A11" s="2"/>
-      <c r="B11" s="2"/>
-      <c r="C11" s="2"/>
-      <c r="D11" s="2"/>
-      <c r="E11" s="2"/>
-      <c r="F11" s="2"/>
+      <c r="A11" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D11" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="E11" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="F11" s="2" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>43</v>
+      </c>
+      <c r="B12" t="s">
+        <v>50</v>
+      </c>
+      <c r="C12" t="s">
+        <v>2</v>
+      </c>
+      <c r="D12" t="s">
+        <v>53</v>
+      </c>
+      <c r="E12" t="s">
+        <v>35</v>
+      </c>
+      <c r="F12" t="s">
+        <v>46</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -677,68 +794,68 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C1" s="3" t="s">
         <v>6</v>
-      </c>
-      <c r="B1" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="C1" s="3" t="s">
-        <v>8</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="B3" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="C3" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="B5" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="C5" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="B6" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="C6" s="2" t="s">
         <v>25</v>
-      </c>
-      <c r="C6" s="2" t="s">
-        <v>28</v>
       </c>
     </row>
   </sheetData>

</xml_diff>